<commit_message>
Update capital structure database
</commit_message>
<xml_diff>
--- a/research/traditional_assets/database/data/anguilla/anguilla_entertainment.xlsx
+++ b/research/traditional_assets/database/data/anguilla/anguilla_entertainment.xlsx
@@ -588,25 +588,25 @@
         </is>
       </c>
       <c r="D2">
-        <v>0.985</v>
+        <v>1.632</v>
       </c>
       <c r="G2">
-        <v>0.2088118811881188</v>
+        <v>0.2302816901408451</v>
       </c>
       <c r="H2">
-        <v>0.05732673267326732</v>
+        <v>0.07042253521126761</v>
       </c>
       <c r="I2">
-        <v>0.0118276207104564</v>
+        <v>-0.02738966474999021</v>
       </c>
       <c r="J2">
-        <v>0.0118276207104564</v>
+        <v>-0.02738966474999021</v>
       </c>
       <c r="K2">
-        <v>-0.215</v>
+        <v>-0.99</v>
       </c>
       <c r="L2">
-        <v>-0.02128712871287129</v>
+        <v>-0.06971830985915493</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -630,55 +630,55 @@
         <v>0</v>
       </c>
       <c r="U2">
-        <v>1.19</v>
+        <v>1.83</v>
       </c>
       <c r="V2">
-        <v>0.01925566343042071</v>
+        <v>0.05366568914956012</v>
       </c>
       <c r="W2">
-        <v>-0.0274234693877551</v>
+        <v>-0.118421052631579</v>
       </c>
       <c r="X2">
-        <v>0.1355242246544866</v>
+        <v>0.2286491947984781</v>
       </c>
       <c r="Y2">
-        <v>-0.1629476940422417</v>
+        <v>-0.347070247430057</v>
       </c>
       <c r="Z2">
-        <v>2.74627779464049</v>
+        <v>3.483238340578712</v>
       </c>
       <c r="AA2">
-        <v>0.0324819321205564</v>
+        <v>-0.09540473039276315</v>
       </c>
       <c r="AB2">
-        <v>0.1352046917068975</v>
+        <v>0.2280455126359717</v>
       </c>
       <c r="AC2">
-        <v>-0.1027227595863411</v>
+        <v>-0.3234502430287349</v>
       </c>
       <c r="AD2">
-        <v>0.047</v>
+        <v>0.044</v>
       </c>
       <c r="AE2">
-        <v>0.2477051541219516</v>
+        <v>0.1596661972493048</v>
       </c>
       <c r="AF2">
-        <v>0.2947051541219516</v>
+        <v>0.2036661972493048</v>
       </c>
       <c r="AG2">
-        <v>-0.8952948458780483</v>
+        <v>-1.626333802750695</v>
       </c>
       <c r="AH2">
-        <v>0.004746059320041535</v>
+        <v>0.005937155407186072</v>
       </c>
       <c r="AI2">
-        <v>0.03405143778717792</v>
+        <v>0.0242642717095479</v>
       </c>
       <c r="AJ2">
-        <v>-0.01469992907136594</v>
+        <v>-0.05008161976144395</v>
       </c>
       <c r="AK2">
-        <v>-0.1199370674920326</v>
+        <v>-0.2477782620073303</v>
       </c>
       <c r="AL2">
         <v>0</v>
@@ -687,10 +687,10 @@
         <v>0</v>
       </c>
       <c r="AN2">
-        <v>0.06403269754768393</v>
+        <v>0.2178217821782178</v>
       </c>
       <c r="AP2">
-        <v>-1.219747746427859</v>
+        <v>-8.051157439359876</v>
       </c>
     </row>
     <row r="3">
@@ -710,25 +710,25 @@
         </is>
       </c>
       <c r="D3">
-        <v>0.985</v>
+        <v>1.632</v>
       </c>
       <c r="G3">
-        <v>0.2088118811881188</v>
+        <v>0.2302816901408451</v>
       </c>
       <c r="H3">
-        <v>0.05732673267326732</v>
+        <v>0.07042253521126761</v>
       </c>
       <c r="I3">
-        <v>0.0118276207104564</v>
+        <v>-0.02738966474999021</v>
       </c>
       <c r="J3">
-        <v>0.0118276207104564</v>
+        <v>-0.02738966474999021</v>
       </c>
       <c r="K3">
-        <v>-0.215</v>
+        <v>-0.99</v>
       </c>
       <c r="L3">
-        <v>-0.02128712871287129</v>
+        <v>-0.06971830985915493</v>
       </c>
       <c r="M3">
         <v>-0</v>
@@ -752,55 +752,55 @@
         <v>0</v>
       </c>
       <c r="U3">
-        <v>1.19</v>
+        <v>1.83</v>
       </c>
       <c r="V3">
-        <v>0.01925566343042071</v>
+        <v>0.05366568914956012</v>
       </c>
       <c r="W3">
-        <v>-0.0274234693877551</v>
+        <v>-0.118421052631579</v>
       </c>
       <c r="X3">
-        <v>0.1355242246544866</v>
+        <v>0.2286491947984781</v>
       </c>
       <c r="Y3">
-        <v>-0.1629476940422417</v>
+        <v>-0.347070247430057</v>
       </c>
       <c r="Z3">
-        <v>2.74627779464049</v>
+        <v>3.483238340578712</v>
       </c>
       <c r="AA3">
-        <v>0.0324819321205564</v>
+        <v>-0.09540473039276315</v>
       </c>
       <c r="AB3">
-        <v>0.1352046917068975</v>
+        <v>0.2280455126359717</v>
       </c>
       <c r="AC3">
-        <v>-0.1027227595863411</v>
+        <v>-0.3234502430287349</v>
       </c>
       <c r="AD3">
-        <v>0.047</v>
+        <v>0.044</v>
       </c>
       <c r="AE3">
-        <v>0.2477051541219516</v>
+        <v>0.1596661972493048</v>
       </c>
       <c r="AF3">
-        <v>0.2947051541219516</v>
+        <v>0.2036661972493048</v>
       </c>
       <c r="AG3">
-        <v>-0.8952948458780483</v>
+        <v>-1.626333802750695</v>
       </c>
       <c r="AH3">
-        <v>0.004746059320041535</v>
+        <v>0.005937155407186072</v>
       </c>
       <c r="AI3">
-        <v>0.03405143778717792</v>
+        <v>0.0242642717095479</v>
       </c>
       <c r="AJ3">
-        <v>-0.01469992907136594</v>
+        <v>-0.05008161976144395</v>
       </c>
       <c r="AK3">
-        <v>-0.1199370674920326</v>
+        <v>-0.2477782620073303</v>
       </c>
       <c r="AL3">
         <v>0</v>
@@ -809,10 +809,10 @@
         <v>0</v>
       </c>
       <c r="AN3">
-        <v>0.06403269754768393</v>
+        <v>0.2178217821782178</v>
       </c>
       <c r="AP3">
-        <v>-1.219747746427859</v>
+        <v>-8.051157439359876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>